<commit_message>
Sesión 3: caso, contenidos y lista de cotejo del bloque de calidad
</commit_message>
<xml_diff>
--- a/03_Entregables-diseño/SI - Ciclo II/1 - SI-SGCSSMA - Sistema de gestión de calidad, seguridad, salud y medio ambiente/03_Matriz-de-distribucion.xlsx
+++ b/03_Entregables-diseño/SI - Ciclo II/1 - SI-SGCSSMA - Sistema de gestión de calidad, seguridad, salud y medio ambiente/03_Matriz-de-distribucion.xlsx
@@ -259,13 +259,13 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="J21" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L21" s="19" t="inlineStr">
         <is>
-          <t>31 láms</t>
+          <t>32 láms</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="J22" s="11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L22" s="19" t="inlineStr">
         <is>
-          <t>28 láms</t>
+          <t>31 láms</t>
         </is>
       </c>
     </row>
@@ -1143,27 +1143,25 @@
           <t>TC1 · c1</t>
         </is>
       </c>
-      <c r="H23" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J23" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K23" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L23" s="26" t="inlineStr">
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>4 pk</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1205,27 +1203,27 @@
           <t>TC1 · c1</t>
         </is>
       </c>
-      <c r="H24" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J24" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K24" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L24" s="26" t="inlineStr">
+      <c r="H24" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L24" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1267,27 +1265,27 @@
           <t>TC1 · c1</t>
         </is>
       </c>
-      <c r="H25" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J25" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K25" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L25" s="26" t="inlineStr">
+      <c r="H25" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1329,27 +1327,27 @@
           <t>TC1 · c1</t>
         </is>
       </c>
-      <c r="H26" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J26" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K26" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L26" s="26" t="inlineStr">
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1391,27 +1389,27 @@
           <t>TC1 · c2</t>
         </is>
       </c>
-      <c r="H27" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="26" t="inlineStr">
+      <c r="H27" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1453,27 +1451,27 @@
           <t>TC1 · c2</t>
         </is>
       </c>
-      <c r="H28" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="26" t="inlineStr">
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1515,27 +1513,27 @@
           <t>TC1 · c2</t>
         </is>
       </c>
-      <c r="H29" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J29" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K29" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L29" s="26" t="inlineStr">
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L29" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1577,27 +1575,27 @@
           <t>TC1 · c2</t>
         </is>
       </c>
-      <c r="H30" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J30" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K30" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L30" s="26" t="inlineStr">
+      <c r="H30" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1763,27 +1761,27 @@
           <t>TC2 · c2</t>
         </is>
       </c>
-      <c r="H33" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J33" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K33" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L33" s="26" t="inlineStr">
+      <c r="H33" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1825,27 +1823,27 @@
           <t>TC2 · c2</t>
         </is>
       </c>
-      <c r="H34" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I34" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J34" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K34" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L34" s="26" t="inlineStr">
+      <c r="H34" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1887,27 +1885,27 @@
           <t>TC2 · c2</t>
         </is>
       </c>
-      <c r="H35" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J35" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K35" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L35" s="26" t="inlineStr">
+      <c r="H35" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1949,27 +1947,27 @@
           <t>TC2 · c1</t>
         </is>
       </c>
-      <c r="H36" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J36" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K36" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L36" s="26" t="inlineStr">
+      <c r="H36" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J36" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K36" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L36" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2011,27 +2009,27 @@
           <t>TC2 · c1</t>
         </is>
       </c>
-      <c r="H37" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I37" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J37" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K37" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L37" s="26" t="inlineStr">
+      <c r="H37" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J37" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L37" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2073,27 +2071,27 @@
           <t>TC2 · c2</t>
         </is>
       </c>
-      <c r="H38" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I38" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J38" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K38" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L38" s="26" t="inlineStr">
+      <c r="H38" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L38" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2135,27 +2133,27 @@
           <t>TC2 · c3</t>
         </is>
       </c>
-      <c r="H39" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J39" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K39" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L39" s="26" t="inlineStr">
+      <c r="H39" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J39" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L39" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2197,27 +2195,27 @@
           <t>TC2 · c3</t>
         </is>
       </c>
-      <c r="H40" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J40" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K40" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L40" s="26" t="inlineStr">
+      <c r="H40" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J40" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2259,27 +2257,27 @@
           <t>TC2 · c3</t>
         </is>
       </c>
-      <c r="H41" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I41" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J41" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K41" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L41" s="26" t="inlineStr">
+      <c r="H41" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J41" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2321,27 +2319,27 @@
           <t>TC2 · c3</t>
         </is>
       </c>
-      <c r="H42" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I42" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J42" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K42" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L42" s="26" t="inlineStr">
+      <c r="H42" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J42" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2506,16 +2504,16 @@
       </c>
       <c r="B48" s="40" t="inlineStr">
         <is>
-          <t>▉▉▉···························</t>
+          <t>▉▉▉▉··························</t>
         </is>
       </c>
       <c r="K48" s="41" t="inlineStr">
         <is>
-          <t>2 de 20</t>
+          <t>3 de 20</t>
         </is>
       </c>
       <c r="L48" s="43" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="49">
@@ -2526,16 +2524,16 @@
       </c>
       <c r="B49" s="40" t="inlineStr">
         <is>
-          <t>▉▉▉···························</t>
+          <t>▉▉▉▉··························</t>
         </is>
       </c>
       <c r="K49" s="41" t="inlineStr">
         <is>
-          <t>2 de 20</t>
+          <t>3 de 20</t>
         </is>
       </c>
       <c r="L49" s="43" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="50">
@@ -2546,16 +2544,16 @@
       </c>
       <c r="B50" s="40" t="inlineStr">
         <is>
-          <t>▉▉▉···························</t>
+          <t>▉▉▉▉··························</t>
         </is>
       </c>
       <c r="K50" s="41" t="inlineStr">
         <is>
-          <t>2 de 20</t>
+          <t>3 de 20</t>
         </is>
       </c>
       <c r="L50" s="43" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="51">
@@ -2566,16 +2564,16 @@
       </c>
       <c r="B51" s="40" t="inlineStr">
         <is>
-          <t>▉▉▉···························</t>
+          <t>▉▉▉▉··························</t>
         </is>
       </c>
       <c r="K51" s="41" t="inlineStr">
         <is>
-          <t>2 de 20</t>
+          <t>3 de 20</t>
         </is>
       </c>
       <c r="L51" s="43" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Caso A y caso B sustituyen a «variante»; revisar_tc lee criterios de varios indicadores
- La palabra «variante» sale del proyecto (H-34): columnas de casos.csv,
  títulos de lámina, §13, §14 y la matriz de distribución. No se tocan los
  tres sitios donde la palabra significa otra cosa.
- revisar_tc.py daba por ajeno un criterio etiquetado «IND-2;IND-3»: leía
  la cadena entera como un indicador inexistente. Ahora separa por «;».
</commit_message>
<xml_diff>
--- a/03_Entregables-diseño/SI - Ciclo II/1 - SI-SGCSSMA - Sistema de gestión de calidad, seguridad, salud y medio ambiente/03_Matriz-de-distribucion.xlsx
+++ b/03_Entregables-diseño/SI - Ciclo II/1 - SI-SGCSSMA - Sistema de gestión de calidad, seguridad, salud y medio ambiente/03_Matriz-de-distribucion.xlsx
@@ -757,7 +757,7 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>indicadores  →  ①TC1 y TC2  →  ②aprendizajes esperados  →  ③2 variantes por sesión  →  ④lista de cotejo  →  ⑤puntos clave  →  ⑥PPT</t>
+          <t>indicadores  →  ①TC1 y TC2  →  ②aprendizajes esperados  →  ③2 casos A y B por sesión  →  ④lista de cotejo  →  ⑤puntos clave  →  ⑥PPT</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
     <row r="48">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>③ Variante A</t>
+          <t>③ Caso A</t>
         </is>
       </c>
       <c r="B48" s="40" t="inlineStr">
@@ -2519,7 +2519,7 @@
     <row r="49">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>③ Variante B</t>
+          <t>③ Caso B</t>
         </is>
       </c>
       <c r="B49" s="40" t="inlineStr">

</xml_diff>